<commit_message>
Add fishing sub-index columns and simplify fishing type categories
Export the marine and inland fishing sub-indices as their own columns, rename them for consistency (Marine/Inland/Highest type), simplify "Fishing type" to show only the higher-scoring type instead of a combined category, and fix the description of the composite index. Propagated to translations and data dictionaries.
</commit_message>
<xml_diff>
--- a/docs/settlements_data_dictionary.xlsx
+++ b/docs/settlements_data_dictionary.xlsx
@@ -1558,11 +1558,15 @@
       <c r="A58" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>98</v>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Fishing Activity (Highest type)</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Composite indicator of fishing activity, taken as the higher of the marine and inland sub-indices (0=lowest, 1=highest).</t>
+        </is>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
@@ -1572,8 +1576,10 @@
       <c r="B59" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C59" s="4" t="s">
-        <v>99</v>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Predominant fishing modality (marine or inland), based on whichever activity sub-index scores higher</t>
+        </is>
       </c>
     </row>
     <row r="60" spans="1:3" ht="25.75" x14ac:dyDescent="0.35">

</xml_diff>